<commit_message>
Filling in array with GetopXsection data now works for all 10 examples.
</commit_message>
<xml_diff>
--- a/Projects/ARK_RWS/data/ARKPropSections.xlsx
+++ b/Projects/ARK_RWS/data/ARKPropSections.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6lab/Projects/ARK-RWS/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Theo/Development/python/mf6_tools/mf6lab/Projects/ARK_RWS/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{67B71577-914F-724B-8B3B-E73F7886E0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AE295C-D7C6-4541-B0B9-1B75DAFE6033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="2280" windowWidth="28040" windowHeight="17180" xr2:uid="{A93E3A23-F585-B641-BD2F-3715E1F34202}"/>
+    <workbookView xWindow="3940" yWindow="3520" windowWidth="28040" windowHeight="17180" xr2:uid="{A93E3A23-F585-B641-BD2F-3715E1F34202}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,6 +33,80 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="23">
+  <si>
+    <t>NUAAOP</t>
+  </si>
+  <si>
+    <t>NUECgb</t>
+  </si>
+  <si>
+    <t>NUEC1</t>
+  </si>
+  <si>
+    <t>NUNIHO</t>
+  </si>
+  <si>
+    <t>NUNIBA</t>
+  </si>
+  <si>
+    <t>NUNBXWI-SI-KO</t>
+  </si>
+  <si>
+    <t>NUBX</t>
+  </si>
+  <si>
+    <t>NUKR-BXDE</t>
+  </si>
+  <si>
+    <t>NUDR</t>
+  </si>
+  <si>
+    <t>Nugs</t>
+  </si>
+  <si>
+    <t>NUUR2</t>
+  </si>
+  <si>
+    <t>NUST</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>kz</t>
+  </si>
+  <si>
+    <t>zf</t>
+  </si>
+  <si>
+    <t>zm</t>
+  </si>
+  <si>
+    <t>zg</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>she</t>
+  </si>
+  <si>
+    <t>NUECga</t>
+  </si>
+  <si>
+    <t>NUgs</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -402,9 +476,690 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C8BD6F-7BA2-8B4C-B07A-BF9D01B40972}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" t="s">
+        <v>3</v>
+      </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" t="s">
+        <v>5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G8" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
+        <v>4</v>
+      </c>
+      <c r="F18" t="s">
+        <v>5</v>
+      </c>
+      <c r="G18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" t="s">
+        <v>7</v>
+      </c>
+      <c r="I18" t="s">
+        <v>8</v>
+      </c>
+      <c r="J18" t="s">
+        <v>9</v>
+      </c>
+      <c r="K18" t="s">
+        <v>10</v>
+      </c>
+      <c r="L18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H20" t="s">
+        <v>19</v>
+      </c>
+      <c r="I20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2</v>
+      </c>
+      <c r="D21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" t="s">
+        <v>6</v>
+      </c>
+      <c r="H21" t="s">
+        <v>7</v>
+      </c>
+      <c r="I21" t="s">
+        <v>8</v>
+      </c>
+      <c r="J21" t="s">
+        <v>22</v>
+      </c>
+      <c r="K21" t="s">
+        <v>10</v>
+      </c>
+      <c r="L21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" t="s">
+        <v>3</v>
+      </c>
+      <c r="F22" t="s">
+        <v>4</v>
+      </c>
+      <c r="G22" t="s">
+        <v>5</v>
+      </c>
+      <c r="H22" t="s">
+        <v>6</v>
+      </c>
+      <c r="I22" t="s">
+        <v>8</v>
+      </c>
+      <c r="J22" t="s">
+        <v>22</v>
+      </c>
+      <c r="K22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>2</v>
+      </c>
+      <c r="E23" t="s">
+        <v>3</v>
+      </c>
+      <c r="F23" t="s">
+        <v>4</v>
+      </c>
+      <c r="G23" t="s">
+        <v>5</v>
+      </c>
+      <c r="H23" t="s">
+        <v>6</v>
+      </c>
+      <c r="I23" t="s">
+        <v>7</v>
+      </c>
+      <c r="J23" t="s">
+        <v>8</v>
+      </c>
+      <c r="K23" t="s">
+        <v>22</v>
+      </c>
+      <c r="L23" t="s">
+        <v>10</v>
+      </c>
+      <c r="M23" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" t="s">
+        <v>4</v>
+      </c>
+      <c r="F24" t="s">
+        <v>5</v>
+      </c>
+      <c r="G24" t="s">
+        <v>6</v>
+      </c>
+      <c r="H24" t="s">
+        <v>7</v>
+      </c>
+      <c r="I24" t="s">
+        <v>8</v>
+      </c>
+      <c r="J24" t="s">
+        <v>22</v>
+      </c>
+      <c r="K24" t="s">
+        <v>10</v>
+      </c>
+      <c r="L24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" t="s">
+        <v>15</v>
+      </c>
+      <c r="E25" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" t="s">
+        <v>18</v>
+      </c>
+      <c r="H25" t="s">
+        <v>19</v>
+      </c>
+      <c r="I25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>12</v>
+      </c>
+      <c r="B26" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" t="s">
+        <v>16</v>
+      </c>
+      <c r="F26" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" t="s">
+        <v>18</v>
+      </c>
+      <c r="H26" t="s">
+        <v>19</v>
+      </c>
+      <c r="I26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>12</v>
+      </c>
+      <c r="B27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E27" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" t="s">
+        <v>18</v>
+      </c>
+      <c r="H27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>